<commit_message>
feat(ai): 落盘action-auth i18n属性与web i18n yaml及模型更新
- 更新nop-ai.orm.xml和ai-gen.orm.xml模型定义

- 更新所有xmeta displayName属性

- 落盘action-auth i18n属性

- 更新en i18n yaml翻译文件

- 更新生成的view.xml文件

- 更新orm.xlsx二进制模型
</commit_message>
<xml_diff>
--- a/nop-ai/nop-ai-coder/demo/model/app-demo.orm.xlsx
+++ b/nop-ai/nop-ai-coder/demo/model/app-demo.orm.xlsx
@@ -183,7 +183,7 @@
     </font>
     <font>
       <name val="等线"/>
-      <u/>
+      <u val="single"/>
       <sz val="11"/>
       <charset val="134"/>
       <family val="2"/>
@@ -1214,14 +1214,14 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0da34220-a9a4-4234-938a-fb0b4f734b6c}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:D9"/>
-  <sheetFormatPr defaultRowHeight="14.0" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5.6640625" customWidth="1"/>
-    <col min="2" max="2" width="19.58203125" customWidth="1"/>
-    <col min="3" max="3" width="19.58203125" customWidth="1"/>
-    <col min="4" max="4" width="16.5" customWidth="1"/>
+    <col min="2" max="2" width="19.5546875" customWidth="1"/>
+    <col min="3" max="3" width="19.5546875" customWidth="1"/>
+    <col min="4" max="4" width="16.44140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
@@ -1304,26 +1304,26 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3c22338c-43ff-4717-adb1-c8735841c492}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:R50"/>
-  <sheetFormatPr defaultRowHeight="14.0" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.33203125" customWidth="1"/>
-    <col min="2" max="2" width="4.4140625" customWidth="1"/>
+    <col min="2" max="2" width="4.44140625" customWidth="1"/>
     <col min="3" max="3" width="5.6640625" customWidth="1"/>
-    <col min="4" max="4" width="12.9140625" customWidth="1"/>
+    <col min="4" max="4" width="12.88671875" customWidth="1"/>
     <col min="5" max="5" width="4.6640625" customWidth="1"/>
-    <col min="6" max="6" width="4.75" customWidth="1"/>
-    <col min="7" max="7" width="15.08203125" customWidth="1"/>
+    <col min="6" max="6" width="4.77734375" customWidth="1"/>
+    <col min="7" max="7" width="15.109375" customWidth="1"/>
     <col min="8" max="8" width="13.0" customWidth="1"/>
     <col min="9" max="9" width="8.5" customWidth="1"/>
-    <col min="10" max="10" width="6.25" customWidth="1"/>
-    <col min="11" max="11" width="4.75" customWidth="1"/>
+    <col min="10" max="10" width="6.21875" customWidth="1"/>
+    <col min="11" max="11" width="4.77734375" customWidth="1"/>
     <col min="12" max="12" width="11.0" customWidth="1"/>
-    <col min="13" max="13" width="6.08203125" customWidth="1"/>
-    <col min="14" max="14" width="8.25" customWidth="1"/>
+    <col min="13" max="13" width="6.109375" customWidth="1"/>
+    <col min="14" max="14" width="8.21875" customWidth="1"/>
     <col min="15" max="15" width="12.6640625" customWidth="1"/>
-    <col min="16" max="16" width="11.08203125" customWidth="1"/>
+    <col min="16" max="16" width="11.109375" customWidth="1"/>
     <col min="17" max="17" width="8.5" customWidth="1"/>
     <col min="18" max="18" width="8.5" customWidth="1"/>
   </cols>
@@ -1409,7 +1409,11 @@
       <c r="F3" s="67"/>
       <c r="G3" s="67"/>
       <c r="H3" s="67"/>
-      <c r="I3" s="5"/>
+      <c r="I3" s="5" t="inlineStr">
+        <is>
+          <t>所属模块</t>
+        </is>
+      </c>
       <c r="J3" s="34"/>
       <c r="K3" s="34"/>
       <c r="L3" s="34"/>
@@ -1515,7 +1519,7 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>属性名</t>
+          <t>控件</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -1599,11 +1603,7 @@
           <t>id</t>
         </is>
       </c>
-      <c r="E8" s="9" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
+      <c r="E8" s="9"/>
       <c r="F8" s="7"/>
       <c r="G8" s="9"/>
       <c r="H8" s="9" t="inlineStr">
@@ -1645,11 +1645,7 @@
           <t>warehouse_name</t>
         </is>
       </c>
-      <c r="E9" s="9" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="E9" s="9"/>
       <c r="F9" s="7"/>
       <c r="G9" s="9"/>
       <c r="H9" s="9" t="inlineStr">
@@ -1691,11 +1687,7 @@
           <t>company_id</t>
         </is>
       </c>
-      <c r="E10" s="9" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="E10" s="9"/>
       <c r="F10" s="7"/>
       <c r="G10" s="9"/>
       <c r="H10" s="9" t="inlineStr">
@@ -1737,11 +1729,7 @@
           <t>remark</t>
         </is>
       </c>
-      <c r="E11" s="9" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="E11" s="9"/>
       <c r="F11" s="7"/>
       <c r="G11" s="9"/>
       <c r="H11" s="9" t="inlineStr">
@@ -1781,11 +1769,7 @@
       </c>
       <c r="C12" s="7"/>
       <c r="D12" s="9"/>
-      <c r="E12" s="9" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="E12" s="9"/>
       <c r="F12" s="7"/>
       <c r="G12" s="9"/>
       <c r="H12" s="9"/>
@@ -1817,11 +1801,7 @@
       </c>
       <c r="C13" s="7"/>
       <c r="D13" s="9"/>
-      <c r="E13" s="9" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="E13" s="9"/>
       <c r="F13" s="7"/>
       <c r="G13" s="9"/>
       <c r="H13" s="9"/>
@@ -2303,9 +2283,7 @@
         </is>
       </c>
       <c r="N28" s="60"/>
-      <c r="O28" s="41" t="b">
-        <v>0</v>
-      </c>
+      <c r="O28" s="41"/>
       <c r="P28" s="41"/>
       <c r="Q28" s="41"/>
       <c r="R28" s="41"/>
@@ -2569,9 +2547,7 @@
         </is>
       </c>
       <c r="N36" s="60"/>
-      <c r="O36" s="41" t="b">
-        <v>0</v>
-      </c>
+      <c r="O36" s="41"/>
       <c r="P36" s="41"/>
       <c r="Q36" s="41"/>
       <c r="R36" s="41"/>
@@ -3120,26 +3096,26 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{89877624-ac0b-4f21-8bba-00a02d6fe6ce}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:R53"/>
-  <sheetFormatPr defaultRowHeight="14.0" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.33203125" customWidth="1"/>
-    <col min="2" max="2" width="4.4140625" customWidth="1"/>
+    <col min="2" max="2" width="4.44140625" customWidth="1"/>
     <col min="3" max="3" width="5.6640625" customWidth="1"/>
-    <col min="4" max="4" width="12.9140625" customWidth="1"/>
+    <col min="4" max="4" width="12.88671875" customWidth="1"/>
     <col min="5" max="5" width="4.6640625" customWidth="1"/>
-    <col min="6" max="6" width="4.75" customWidth="1"/>
-    <col min="7" max="7" width="15.08203125" customWidth="1"/>
+    <col min="6" max="6" width="4.77734375" customWidth="1"/>
+    <col min="7" max="7" width="15.109375" customWidth="1"/>
     <col min="8" max="8" width="13.0" customWidth="1"/>
     <col min="9" max="9" width="8.5" customWidth="1"/>
-    <col min="10" max="10" width="6.25" customWidth="1"/>
-    <col min="11" max="11" width="4.75" customWidth="1"/>
+    <col min="10" max="10" width="6.21875" customWidth="1"/>
+    <col min="11" max="11" width="4.77734375" customWidth="1"/>
     <col min="12" max="12" width="11.0" customWidth="1"/>
-    <col min="13" max="13" width="6.08203125" customWidth="1"/>
-    <col min="14" max="14" width="8.25" customWidth="1"/>
+    <col min="13" max="13" width="6.109375" customWidth="1"/>
+    <col min="14" max="14" width="8.21875" customWidth="1"/>
     <col min="15" max="15" width="12.6640625" customWidth="1"/>
-    <col min="16" max="16" width="11.08203125" customWidth="1"/>
+    <col min="16" max="16" width="11.109375" customWidth="1"/>
     <col min="17" max="17" width="8.5" customWidth="1"/>
     <col min="18" max="18" width="8.5" customWidth="1"/>
   </cols>
@@ -3225,7 +3201,11 @@
       <c r="F3" s="67"/>
       <c r="G3" s="67"/>
       <c r="H3" s="67"/>
-      <c r="I3" s="5"/>
+      <c r="I3" s="5" t="inlineStr">
+        <is>
+          <t>所属模块</t>
+        </is>
+      </c>
       <c r="J3" s="34"/>
       <c r="K3" s="34"/>
       <c r="L3" s="34"/>
@@ -3331,7 +3311,7 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>属性名</t>
+          <t>控件</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -3415,11 +3395,7 @@
           <t>id</t>
         </is>
       </c>
-      <c r="E8" s="9" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
+      <c r="E8" s="9"/>
       <c r="F8" s="7"/>
       <c r="G8" s="9"/>
       <c r="H8" s="9" t="inlineStr">
@@ -3461,11 +3437,7 @@
           <t>stock_date</t>
         </is>
       </c>
-      <c r="E9" s="9" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="E9" s="9"/>
       <c r="F9" s="7"/>
       <c r="G9" s="9"/>
       <c r="H9" s="9" t="inlineStr">
@@ -3507,11 +3479,7 @@
           <t>warehouse_id</t>
         </is>
       </c>
-      <c r="E10" s="9" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="E10" s="9"/>
       <c r="F10" s="7"/>
       <c r="G10" s="9"/>
       <c r="H10" s="9" t="inlineStr">
@@ -3553,11 +3521,7 @@
           <t>handler</t>
         </is>
       </c>
-      <c r="E11" s="9" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="E11" s="9"/>
       <c r="F11" s="7"/>
       <c r="G11" s="9"/>
       <c r="H11" s="9" t="inlineStr">
@@ -3599,11 +3563,7 @@
           <t>supplier_id</t>
         </is>
       </c>
-      <c r="E12" s="9" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="E12" s="9"/>
       <c r="F12" s="7"/>
       <c r="G12" s="9"/>
       <c r="H12" s="9" t="inlineStr">
@@ -3645,11 +3605,7 @@
           <t>paid_amount</t>
         </is>
       </c>
-      <c r="E13" s="9" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="E13" s="9"/>
       <c r="F13" s="7"/>
       <c r="G13" s="9"/>
       <c r="H13" s="9" t="inlineStr">
@@ -3695,11 +3651,7 @@
           <t>total_amount</t>
         </is>
       </c>
-      <c r="E14" s="9" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="E14" s="9"/>
       <c r="F14" s="7"/>
       <c r="G14" s="9"/>
       <c r="H14" s="9" t="inlineStr">
@@ -3745,11 +3697,7 @@
           <t>attachments</t>
         </is>
       </c>
-      <c r="E15" s="9" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="E15" s="9"/>
       <c r="F15" s="7"/>
       <c r="G15" s="9"/>
       <c r="H15" s="9" t="inlineStr">
@@ -3791,11 +3739,7 @@
           <t>stock_type</t>
         </is>
       </c>
-      <c r="E16" s="9" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="E16" s="9"/>
       <c r="F16" s="7"/>
       <c r="G16" s="9"/>
       <c r="H16" s="9" t="inlineStr">
@@ -4555,9 +4499,7 @@
         </is>
       </c>
       <c r="N39" s="60"/>
-      <c r="O39" s="41" t="b">
-        <v>0</v>
-      </c>
+      <c r="O39" s="41"/>
       <c r="P39" s="41"/>
       <c r="Q39" s="41"/>
       <c r="R39" s="41"/>
@@ -5106,26 +5048,26 @@
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6984cc15-4aec-454e-8584-3cc8f8869059}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:R45"/>
-  <sheetFormatPr defaultRowHeight="14.0" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.33203125" customWidth="1"/>
-    <col min="2" max="2" width="4.4140625" customWidth="1"/>
+    <col min="2" max="2" width="4.44140625" customWidth="1"/>
     <col min="3" max="3" width="5.6640625" customWidth="1"/>
-    <col min="4" max="4" width="12.9140625" customWidth="1"/>
+    <col min="4" max="4" width="12.88671875" customWidth="1"/>
     <col min="5" max="5" width="4.6640625" customWidth="1"/>
-    <col min="6" max="6" width="4.75" customWidth="1"/>
-    <col min="7" max="7" width="15.08203125" customWidth="1"/>
+    <col min="6" max="6" width="4.77734375" customWidth="1"/>
+    <col min="7" max="7" width="15.109375" customWidth="1"/>
     <col min="8" max="8" width="13.0" customWidth="1"/>
     <col min="9" max="9" width="8.5" customWidth="1"/>
-    <col min="10" max="10" width="6.25" customWidth="1"/>
-    <col min="11" max="11" width="4.75" customWidth="1"/>
+    <col min="10" max="10" width="6.21875" customWidth="1"/>
+    <col min="11" max="11" width="4.77734375" customWidth="1"/>
     <col min="12" max="12" width="11.0" customWidth="1"/>
-    <col min="13" max="13" width="6.08203125" customWidth="1"/>
-    <col min="14" max="14" width="8.25" customWidth="1"/>
+    <col min="13" max="13" width="6.109375" customWidth="1"/>
+    <col min="14" max="14" width="8.21875" customWidth="1"/>
     <col min="15" max="15" width="12.6640625" customWidth="1"/>
-    <col min="16" max="16" width="11.08203125" customWidth="1"/>
+    <col min="16" max="16" width="11.109375" customWidth="1"/>
     <col min="17" max="17" width="8.5" customWidth="1"/>
     <col min="18" max="18" width="8.5" customWidth="1"/>
   </cols>
@@ -5211,7 +5153,11 @@
       <c r="F3" s="67"/>
       <c r="G3" s="67"/>
       <c r="H3" s="67"/>
-      <c r="I3" s="5"/>
+      <c r="I3" s="5" t="inlineStr">
+        <is>
+          <t>所属模块</t>
+        </is>
+      </c>
       <c r="J3" s="34"/>
       <c r="K3" s="34"/>
       <c r="L3" s="34"/>
@@ -5317,7 +5263,7 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>属性名</t>
+          <t>控件</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -5401,11 +5347,7 @@
           <t>id</t>
         </is>
       </c>
-      <c r="E8" s="9" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
+      <c r="E8" s="9"/>
       <c r="F8" s="7"/>
       <c r="G8" s="9"/>
       <c r="H8" s="9" t="inlineStr">
@@ -5447,11 +5389,7 @@
           <t>material_id</t>
         </is>
       </c>
-      <c r="E9" s="9" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="E9" s="9"/>
       <c r="F9" s="7"/>
       <c r="G9" s="9"/>
       <c r="H9" s="9" t="inlineStr">
@@ -5493,11 +5431,7 @@
           <t>material_name</t>
         </is>
       </c>
-      <c r="E10" s="9" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="E10" s="9"/>
       <c r="F10" s="7"/>
       <c r="G10" s="9"/>
       <c r="H10" s="9" t="inlineStr">
@@ -5539,11 +5473,7 @@
           <t>specification</t>
         </is>
       </c>
-      <c r="E11" s="9" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="E11" s="9"/>
       <c r="F11" s="7"/>
       <c r="G11" s="9"/>
       <c r="H11" s="9" t="inlineStr">
@@ -5585,11 +5515,7 @@
           <t>unit</t>
         </is>
       </c>
-      <c r="E12" s="9" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="E12" s="9"/>
       <c r="F12" s="7"/>
       <c r="G12" s="9"/>
       <c r="H12" s="9" t="inlineStr">
@@ -5635,11 +5561,7 @@
           <t>unit_price</t>
         </is>
       </c>
-      <c r="E13" s="9" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="E13" s="9"/>
       <c r="F13" s="7"/>
       <c r="G13" s="9"/>
       <c r="H13" s="9" t="inlineStr">
@@ -5685,11 +5607,7 @@
           <t>quantity</t>
         </is>
       </c>
-      <c r="E14" s="9" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="E14" s="9"/>
       <c r="F14" s="7"/>
       <c r="G14" s="9"/>
       <c r="H14" s="9" t="inlineStr">
@@ -5735,11 +5653,7 @@
           <t>amount</t>
         </is>
       </c>
-      <c r="E15" s="9" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="E15" s="9"/>
       <c r="F15" s="7"/>
       <c r="G15" s="9"/>
       <c r="H15" s="9" t="inlineStr">
@@ -5785,11 +5699,7 @@
           <t>in_out_stock_id</t>
         </is>
       </c>
-      <c r="E16" s="9" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="E16" s="9"/>
       <c r="F16" s="7"/>
       <c r="G16" s="9"/>
       <c r="H16" s="9" t="inlineStr">
@@ -6793,26 +6703,26 @@
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{06b8eb2b-895d-498d-8089-79a9e1c9e03a}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:R34"/>
-  <sheetFormatPr defaultRowHeight="14.0" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.33203125" customWidth="1"/>
-    <col min="2" max="2" width="4.4140625" customWidth="1"/>
+    <col min="2" max="2" width="4.44140625" customWidth="1"/>
     <col min="3" max="3" width="5.6640625" customWidth="1"/>
-    <col min="4" max="4" width="12.9140625" customWidth="1"/>
+    <col min="4" max="4" width="12.88671875" customWidth="1"/>
     <col min="5" max="5" width="4.6640625" customWidth="1"/>
-    <col min="6" max="6" width="4.75" customWidth="1"/>
-    <col min="7" max="7" width="15.08203125" customWidth="1"/>
+    <col min="6" max="6" width="4.77734375" customWidth="1"/>
+    <col min="7" max="7" width="15.109375" customWidth="1"/>
     <col min="8" max="8" width="13.0" customWidth="1"/>
     <col min="9" max="9" width="8.5" customWidth="1"/>
-    <col min="10" max="10" width="6.25" customWidth="1"/>
-    <col min="11" max="11" width="4.75" customWidth="1"/>
+    <col min="10" max="10" width="6.21875" customWidth="1"/>
+    <col min="11" max="11" width="4.77734375" customWidth="1"/>
     <col min="12" max="12" width="11.0" customWidth="1"/>
-    <col min="13" max="13" width="6.08203125" customWidth="1"/>
-    <col min="14" max="14" width="8.25" customWidth="1"/>
+    <col min="13" max="13" width="6.109375" customWidth="1"/>
+    <col min="14" max="14" width="8.21875" customWidth="1"/>
     <col min="15" max="15" width="12.6640625" customWidth="1"/>
-    <col min="16" max="16" width="11.08203125" customWidth="1"/>
+    <col min="16" max="16" width="11.109375" customWidth="1"/>
     <col min="17" max="17" width="8.5" customWidth="1"/>
     <col min="18" max="18" width="8.5" customWidth="1"/>
   </cols>
@@ -6898,7 +6808,11 @@
       <c r="F3" s="67"/>
       <c r="G3" s="67"/>
       <c r="H3" s="67"/>
-      <c r="I3" s="5"/>
+      <c r="I3" s="5" t="inlineStr">
+        <is>
+          <t>所属模块</t>
+        </is>
+      </c>
       <c r="J3" s="34"/>
       <c r="K3" s="34"/>
       <c r="L3" s="34"/>
@@ -7004,7 +6918,7 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>属性名</t>
+          <t>控件</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -7088,11 +7002,7 @@
           <t>id</t>
         </is>
       </c>
-      <c r="E8" s="9" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
+      <c r="E8" s="9"/>
       <c r="F8" s="7"/>
       <c r="G8" s="9"/>
       <c r="H8" s="9" t="inlineStr">
@@ -7134,11 +7044,7 @@
           <t>check_date</t>
         </is>
       </c>
-      <c r="E9" s="9" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="E9" s="9"/>
       <c r="F9" s="7"/>
       <c r="G9" s="9"/>
       <c r="H9" s="9" t="inlineStr">
@@ -7180,11 +7086,7 @@
           <t>warehouse_id</t>
         </is>
       </c>
-      <c r="E10" s="9" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="E10" s="9"/>
       <c r="F10" s="7"/>
       <c r="G10" s="9"/>
       <c r="H10" s="9" t="inlineStr">
@@ -7226,11 +7128,7 @@
           <t>handler</t>
         </is>
       </c>
-      <c r="E11" s="9" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="E11" s="9"/>
       <c r="F11" s="7"/>
       <c r="G11" s="9"/>
       <c r="H11" s="9" t="inlineStr">
@@ -7272,11 +7170,7 @@
           <t>check_type</t>
         </is>
       </c>
-      <c r="E12" s="9" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="E12" s="9"/>
       <c r="F12" s="7"/>
       <c r="G12" s="9"/>
       <c r="H12" s="9" t="inlineStr">
@@ -7322,11 +7216,7 @@
           <t>difference_amount</t>
         </is>
       </c>
-      <c r="E13" s="9" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="E13" s="9"/>
       <c r="F13" s="7"/>
       <c r="G13" s="9"/>
       <c r="H13" s="9" t="inlineStr">
@@ -8031,26 +7921,26 @@
 </file>
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{c9f66911-c255-4a51-8f78-ef537ffb8e0b}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:R34"/>
-  <sheetFormatPr defaultRowHeight="14.0" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.33203125" customWidth="1"/>
-    <col min="2" max="2" width="4.4140625" customWidth="1"/>
+    <col min="2" max="2" width="4.44140625" customWidth="1"/>
     <col min="3" max="3" width="5.6640625" customWidth="1"/>
-    <col min="4" max="4" width="12.9140625" customWidth="1"/>
+    <col min="4" max="4" width="12.88671875" customWidth="1"/>
     <col min="5" max="5" width="4.6640625" customWidth="1"/>
-    <col min="6" max="6" width="4.75" customWidth="1"/>
-    <col min="7" max="7" width="15.08203125" customWidth="1"/>
+    <col min="6" max="6" width="4.77734375" customWidth="1"/>
+    <col min="7" max="7" width="15.109375" customWidth="1"/>
     <col min="8" max="8" width="13.0" customWidth="1"/>
     <col min="9" max="9" width="8.5" customWidth="1"/>
-    <col min="10" max="10" width="6.25" customWidth="1"/>
-    <col min="11" max="11" width="4.75" customWidth="1"/>
+    <col min="10" max="10" width="6.21875" customWidth="1"/>
+    <col min="11" max="11" width="4.77734375" customWidth="1"/>
     <col min="12" max="12" width="11.0" customWidth="1"/>
-    <col min="13" max="13" width="6.08203125" customWidth="1"/>
-    <col min="14" max="14" width="8.25" customWidth="1"/>
+    <col min="13" max="13" width="6.109375" customWidth="1"/>
+    <col min="14" max="14" width="8.21875" customWidth="1"/>
     <col min="15" max="15" width="12.6640625" customWidth="1"/>
-    <col min="16" max="16" width="11.08203125" customWidth="1"/>
+    <col min="16" max="16" width="11.109375" customWidth="1"/>
     <col min="17" max="17" width="8.5" customWidth="1"/>
     <col min="18" max="18" width="8.5" customWidth="1"/>
   </cols>
@@ -8136,7 +8026,11 @@
       <c r="F3" s="67"/>
       <c r="G3" s="67"/>
       <c r="H3" s="67"/>
-      <c r="I3" s="5"/>
+      <c r="I3" s="5" t="inlineStr">
+        <is>
+          <t>所属模块</t>
+        </is>
+      </c>
       <c r="J3" s="34"/>
       <c r="K3" s="34"/>
       <c r="L3" s="34"/>
@@ -8242,7 +8136,7 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>属性名</t>
+          <t>控件</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -8326,11 +8220,7 @@
           <t>id</t>
         </is>
       </c>
-      <c r="E8" s="9" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
+      <c r="E8" s="9"/>
       <c r="F8" s="7"/>
       <c r="G8" s="9"/>
       <c r="H8" s="9" t="inlineStr">
@@ -8372,11 +8262,7 @@
           <t>company_id</t>
         </is>
       </c>
-      <c r="E9" s="9" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="E9" s="9"/>
       <c r="F9" s="7"/>
       <c r="G9" s="9"/>
       <c r="H9" s="9" t="inlineStr">
@@ -8418,11 +8304,7 @@
           <t>order_count</t>
         </is>
       </c>
-      <c r="E10" s="9" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="E10" s="9"/>
       <c r="F10" s="7"/>
       <c r="G10" s="9"/>
       <c r="H10" s="9" t="inlineStr">
@@ -8464,11 +8346,7 @@
           <t>operating_cost</t>
         </is>
       </c>
-      <c r="E11" s="9" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="E11" s="9"/>
       <c r="F11" s="7"/>
       <c r="G11" s="9"/>
       <c r="H11" s="9" t="inlineStr">
@@ -8514,11 +8392,7 @@
           <t>daily_deviation</t>
         </is>
       </c>
-      <c r="E12" s="9" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="E12" s="9"/>
       <c r="F12" s="7"/>
       <c r="G12" s="9"/>
       <c r="H12" s="9" t="inlineStr">
@@ -8562,11 +8436,7 @@
       </c>
       <c r="C13" s="7"/>
       <c r="D13" s="9"/>
-      <c r="E13" s="9" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="E13" s="9"/>
       <c r="F13" s="7"/>
       <c r="G13" s="9"/>
       <c r="H13" s="9"/>
@@ -9259,13 +9129,13 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0287e431-1045-425b-bd74-84fa6a17efc8}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:C16"/>
-  <sheetFormatPr defaultRowHeight="14.0" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="22.08203125" customWidth="1"/>
-    <col min="2" max="2" width="27.9140625" customWidth="1"/>
-    <col min="3" max="3" width="39.25" customWidth="1"/>
+    <col min="1" max="1" width="22.109375" customWidth="1"/>
+    <col min="2" max="2" width="27.88671875" customWidth="1"/>
+    <col min="3" max="3" width="39.21875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
@@ -9454,15 +9324,15 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{cd9db001-1c8e-4c1a-aee1-4593e0f37bb4}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:G19"/>
-  <sheetFormatPr defaultRowHeight="14.0" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="4.9140625" customWidth="1"/>
+    <col min="1" max="1" width="4.88671875" customWidth="1"/>
     <col min="2" max="2" width="8.5" customWidth="1"/>
     <col min="3" max="3" width="8.5" customWidth="1"/>
     <col min="4" max="4" width="8.5" customWidth="1"/>
-    <col min="5" max="5" width="9.1640625" customWidth="1"/>
+    <col min="5" max="5" width="9.109375" customWidth="1"/>
     <col min="6" max="6" width="8.5" customWidth="1"/>
     <col min="7" max="7" width="8.5" customWidth="1"/>
   </cols>
@@ -9740,11 +9610,11 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{35910201-2606-4793-b2a8-df844f984ed7}">
-  <dimension ref="A1:G13"/>
-  <sheetFormatPr defaultRowHeight="14.0" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1:G88"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="6.08203125" customWidth="1"/>
+    <col min="1" max="1" width="6.109375" customWidth="1"/>
     <col min="2" max="2" width="8.5" customWidth="1"/>
     <col min="3" max="3" width="8.5" customWidth="1"/>
     <col min="4" max="4" width="8.5" customWidth="1"/>
@@ -9754,14 +9624,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A1" s="29"/>
+      <c r="A1" s="29" t="n">
+        <v>1</v>
+      </c>
       <c r="B1" s="32" t="inlineStr">
         <is>
           <t>名称</t>
         </is>
       </c>
       <c r="C1" s="32"/>
-      <c r="D1" s="34"/>
+      <c r="D1" s="34" t="inlineStr">
+        <is>
+          <t>materialUnit</t>
+        </is>
+      </c>
       <c r="E1" s="34"/>
       <c r="F1" s="20" t="inlineStr">
         <is>
@@ -9778,7 +9654,11 @@
         </is>
       </c>
       <c r="C2" s="32"/>
-      <c r="D2" s="34"/>
+      <c r="D2" s="34" t="inlineStr">
+        <is>
+          <t>计量单位</t>
+        </is>
+      </c>
       <c r="E2" s="34"/>
       <c r="F2" s="20" t="inlineStr">
         <is>
@@ -9795,7 +9675,11 @@
         </is>
       </c>
       <c r="C3" s="32"/>
-      <c r="D3" s="34"/>
+      <c r="D3" s="34" t="inlineStr">
+        <is>
+          <t>计量单位</t>
+        </is>
+      </c>
       <c r="E3" s="34"/>
       <c r="F3" s="34"/>
       <c r="G3" s="34"/>
@@ -9848,39 +9732,111 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="29"/>
-      <c r="B6" s="21"/>
-      <c r="C6" s="21"/>
-      <c r="D6" s="24"/>
-      <c r="E6" s="24"/>
+      <c r="B6" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="C6" s="21" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="D6" s="24" t="inlineStr">
+        <is>
+          <t>千克</t>
+        </is>
+      </c>
+      <c r="E6" s="24" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
       <c r="F6" s="24"/>
-      <c r="G6" s="24"/>
+      <c r="G6" s="24" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="29"/>
-      <c r="B7" s="21"/>
-      <c r="C7" s="21"/>
-      <c r="D7" s="24"/>
-      <c r="E7" s="24"/>
+      <c r="B7" s="21" t="n">
+        <v>2</v>
+      </c>
+      <c r="C7" s="21" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="D7" s="24" t="inlineStr">
+        <is>
+          <t>克</t>
+        </is>
+      </c>
+      <c r="E7" s="24" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
       <c r="F7" s="24"/>
-      <c r="G7" s="24"/>
+      <c r="G7" s="24" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="29"/>
-      <c r="B8" s="21"/>
-      <c r="C8" s="21"/>
-      <c r="D8" s="24"/>
-      <c r="E8" s="24"/>
+      <c r="B8" s="21" t="n">
+        <v>3</v>
+      </c>
+      <c r="C8" s="21" t="inlineStr">
+        <is>
+          <t>piece</t>
+        </is>
+      </c>
+      <c r="D8" s="24" t="inlineStr">
+        <is>
+          <t>个</t>
+        </is>
+      </c>
+      <c r="E8" s="24" t="inlineStr">
+        <is>
+          <t>PIECE</t>
+        </is>
+      </c>
       <c r="F8" s="24"/>
-      <c r="G8" s="24"/>
+      <c r="G8" s="24" t="inlineStr">
+        <is>
+          <t>piece</t>
+        </is>
+      </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="29"/>
-      <c r="B9" s="21"/>
-      <c r="C9" s="21"/>
-      <c r="D9" s="24"/>
-      <c r="E9" s="24"/>
+      <c r="B9" s="21" t="n">
+        <v>4</v>
+      </c>
+      <c r="C9" s="21" t="inlineStr">
+        <is>
+          <t>box</t>
+        </is>
+      </c>
+      <c r="D9" s="24" t="inlineStr">
+        <is>
+          <t>箱</t>
+        </is>
+      </c>
+      <c r="E9" s="24" t="inlineStr">
+        <is>
+          <t>BOX</t>
+        </is>
+      </c>
       <c r="F9" s="24"/>
-      <c r="G9" s="24"/>
+      <c r="G9" s="24" t="inlineStr">
+        <is>
+          <t>box</t>
+        </is>
+      </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="29"/>
@@ -9903,7 +9859,7 @@
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" s="29"/>
       <c r="B12" s="21"/>
-      <c r="C12" s="25"/>
+      <c r="C12" s="21"/>
       <c r="D12" s="24"/>
       <c r="E12" s="24"/>
       <c r="F12" s="24"/>
@@ -9911,16 +9867,1217 @@
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" s="29"/>
-      <c r="B13" s="26"/>
-      <c r="C13" s="26"/>
-      <c r="D13" s="26"/>
-      <c r="E13" s="26"/>
-      <c r="F13" s="26"/>
-      <c r="G13" s="26"/>
+      <c r="B13" s="21"/>
+      <c r="C13" s="21"/>
+      <c r="D13" s="24"/>
+      <c r="E13" s="24"/>
+      <c r="F13" s="24"/>
+      <c r="G13" s="24"/>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A14" s="29"/>
+      <c r="B14" s="21"/>
+      <c r="C14" s="21"/>
+      <c r="D14" s="24"/>
+      <c r="E14" s="24"/>
+      <c r="F14" s="24"/>
+      <c r="G14" s="24"/>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A15" s="29"/>
+      <c r="B15" s="21"/>
+      <c r="C15" s="25"/>
+      <c r="D15" s="24"/>
+      <c r="E15" s="24"/>
+      <c r="F15" s="24"/>
+      <c r="G15" s="24"/>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A16" s="29"/>
+      <c r="B16" s="26"/>
+      <c r="C16" s="26"/>
+      <c r="D16" s="26"/>
+      <c r="E16" s="26"/>
+      <c r="F16" s="26"/>
+      <c r="G16" s="26"/>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A17" s="29" t="n">
+        <v>2</v>
+      </c>
+      <c r="B17" s="32" t="inlineStr">
+        <is>
+          <t>名称</t>
+        </is>
+      </c>
+      <c r="C17" s="32"/>
+      <c r="D17" s="34" t="inlineStr">
+        <is>
+          <t>menuType</t>
+        </is>
+      </c>
+      <c r="E17" s="34"/>
+      <c r="F17" s="20" t="inlineStr">
+        <is>
+          <t>值类型</t>
+        </is>
+      </c>
+      <c r="G17" s="17"/>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A18" s="29"/>
+      <c r="B18" s="32" t="inlineStr">
+        <is>
+          <t>中文名</t>
+        </is>
+      </c>
+      <c r="C18" s="32"/>
+      <c r="D18" s="34" t="inlineStr">
+        <is>
+          <t>菜单类型</t>
+        </is>
+      </c>
+      <c r="E18" s="34"/>
+      <c r="F18" s="20" t="inlineStr">
+        <is>
+          <t>英文名</t>
+        </is>
+      </c>
+      <c r="G18" s="21"/>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A19" s="29"/>
+      <c r="B19" s="32" t="inlineStr">
+        <is>
+          <t>描述</t>
+        </is>
+      </c>
+      <c r="C19" s="32"/>
+      <c r="D19" s="34" t="inlineStr">
+        <is>
+          <t>菜单类型</t>
+        </is>
+      </c>
+      <c r="E19" s="34"/>
+      <c r="F19" s="34"/>
+      <c r="G19" s="34"/>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A20" s="29"/>
+      <c r="B20" s="37" t="inlineStr">
+        <is>
+          <t>字典项</t>
+        </is>
+      </c>
+      <c r="C20" s="37"/>
+      <c r="D20" s="37"/>
+      <c r="E20" s="37"/>
+      <c r="F20" s="37"/>
+      <c r="G20" s="37"/>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A21" s="29"/>
+      <c r="B21" s="22" t="inlineStr">
+        <is>
+          <t>序号</t>
+        </is>
+      </c>
+      <c r="C21" s="23" t="inlineStr">
+        <is>
+          <t>值</t>
+        </is>
+      </c>
+      <c r="D21" s="23" t="inlineStr">
+        <is>
+          <t>名称</t>
+        </is>
+      </c>
+      <c r="E21" s="23" t="inlineStr">
+        <is>
+          <t>代码</t>
+        </is>
+      </c>
+      <c r="F21" s="23" t="inlineStr">
+        <is>
+          <t>英文名</t>
+        </is>
+      </c>
+      <c r="G21" s="23" t="inlineStr">
+        <is>
+          <t>描述</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A22" s="29"/>
+      <c r="B22" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="C22" s="21" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="D22" s="24" t="inlineStr">
+        <is>
+          <t>主食</t>
+        </is>
+      </c>
+      <c r="E22" s="24" t="inlineStr">
+        <is>
+          <t>MAIN</t>
+        </is>
+      </c>
+      <c r="F22" s="24"/>
+      <c r="G22" s="24" t="inlineStr">
+        <is>
+          <t>主食</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A23" s="29"/>
+      <c r="B23" s="21" t="n">
+        <v>2</v>
+      </c>
+      <c r="C23" s="21" t="inlineStr">
+        <is>
+          <t>side</t>
+        </is>
+      </c>
+      <c r="D23" s="24" t="inlineStr">
+        <is>
+          <t>配菜</t>
+        </is>
+      </c>
+      <c r="E23" s="24" t="inlineStr">
+        <is>
+          <t>SIDE</t>
+        </is>
+      </c>
+      <c r="F23" s="24"/>
+      <c r="G23" s="24" t="inlineStr">
+        <is>
+          <t>配菜</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A24" s="29"/>
+      <c r="B24" s="21" t="n">
+        <v>3</v>
+      </c>
+      <c r="C24" s="21" t="inlineStr">
+        <is>
+          <t>drink</t>
+        </is>
+      </c>
+      <c r="D24" s="24" t="inlineStr">
+        <is>
+          <t>饮料</t>
+        </is>
+      </c>
+      <c r="E24" s="24" t="inlineStr">
+        <is>
+          <t>DRINK</t>
+        </is>
+      </c>
+      <c r="F24" s="24"/>
+      <c r="G24" s="24" t="inlineStr">
+        <is>
+          <t>饮料</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A25" s="29"/>
+      <c r="B25" s="21"/>
+      <c r="C25" s="21"/>
+      <c r="D25" s="24"/>
+      <c r="E25" s="24"/>
+      <c r="F25" s="24"/>
+      <c r="G25" s="24"/>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A26" s="29"/>
+      <c r="B26" s="21"/>
+      <c r="C26" s="21"/>
+      <c r="D26" s="24"/>
+      <c r="E26" s="24"/>
+      <c r="F26" s="24"/>
+      <c r="G26" s="24"/>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A27" s="29"/>
+      <c r="B27" s="21"/>
+      <c r="C27" s="21"/>
+      <c r="D27" s="24"/>
+      <c r="E27" s="24"/>
+      <c r="F27" s="24"/>
+      <c r="G27" s="24"/>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A28" s="29"/>
+      <c r="B28" s="21"/>
+      <c r="C28" s="21"/>
+      <c r="D28" s="24"/>
+      <c r="E28" s="24"/>
+      <c r="F28" s="24"/>
+      <c r="G28" s="24"/>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A29" s="29"/>
+      <c r="B29" s="21"/>
+      <c r="C29" s="21"/>
+      <c r="D29" s="24"/>
+      <c r="E29" s="24"/>
+      <c r="F29" s="24"/>
+      <c r="G29" s="24"/>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A30" s="29"/>
+      <c r="B30" s="21"/>
+      <c r="C30" s="25"/>
+      <c r="D30" s="24"/>
+      <c r="E30" s="24"/>
+      <c r="F30" s="24"/>
+      <c r="G30" s="24"/>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A31" s="29"/>
+      <c r="B31" s="26"/>
+      <c r="C31" s="26"/>
+      <c r="D31" s="26"/>
+      <c r="E31" s="26"/>
+      <c r="F31" s="26"/>
+      <c r="G31" s="26"/>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A32" s="29" t="n">
+        <v>3</v>
+      </c>
+      <c r="B32" s="32" t="inlineStr">
+        <is>
+          <t>名称</t>
+        </is>
+      </c>
+      <c r="C32" s="32"/>
+      <c r="D32" s="34" t="inlineStr">
+        <is>
+          <t>stockType</t>
+        </is>
+      </c>
+      <c r="E32" s="34"/>
+      <c r="F32" s="20" t="inlineStr">
+        <is>
+          <t>值类型</t>
+        </is>
+      </c>
+      <c r="G32" s="17"/>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A33" s="29"/>
+      <c r="B33" s="32" t="inlineStr">
+        <is>
+          <t>中文名</t>
+        </is>
+      </c>
+      <c r="C33" s="32"/>
+      <c r="D33" s="34" t="inlineStr">
+        <is>
+          <t>出入库类型</t>
+        </is>
+      </c>
+      <c r="E33" s="34"/>
+      <c r="F33" s="20" t="inlineStr">
+        <is>
+          <t>英文名</t>
+        </is>
+      </c>
+      <c r="G33" s="21"/>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A34" s="29"/>
+      <c r="B34" s="32" t="inlineStr">
+        <is>
+          <t>描述</t>
+        </is>
+      </c>
+      <c r="C34" s="32"/>
+      <c r="D34" s="34" t="inlineStr">
+        <is>
+          <t>出入库类型</t>
+        </is>
+      </c>
+      <c r="E34" s="34"/>
+      <c r="F34" s="34"/>
+      <c r="G34" s="34"/>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A35" s="29"/>
+      <c r="B35" s="37" t="inlineStr">
+        <is>
+          <t>字典项</t>
+        </is>
+      </c>
+      <c r="C35" s="37"/>
+      <c r="D35" s="37"/>
+      <c r="E35" s="37"/>
+      <c r="F35" s="37"/>
+      <c r="G35" s="37"/>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A36" s="29"/>
+      <c r="B36" s="22" t="inlineStr">
+        <is>
+          <t>序号</t>
+        </is>
+      </c>
+      <c r="C36" s="23" t="inlineStr">
+        <is>
+          <t>值</t>
+        </is>
+      </c>
+      <c r="D36" s="23" t="inlineStr">
+        <is>
+          <t>名称</t>
+        </is>
+      </c>
+      <c r="E36" s="23" t="inlineStr">
+        <is>
+          <t>代码</t>
+        </is>
+      </c>
+      <c r="F36" s="23" t="inlineStr">
+        <is>
+          <t>英文名</t>
+        </is>
+      </c>
+      <c r="G36" s="23" t="inlineStr">
+        <is>
+          <t>描述</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A37" s="29"/>
+      <c r="B37" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="C37" s="21" t="inlineStr">
+        <is>
+          <t>in</t>
+        </is>
+      </c>
+      <c r="D37" s="24" t="inlineStr">
+        <is>
+          <t>入库</t>
+        </is>
+      </c>
+      <c r="E37" s="24" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="F37" s="24"/>
+      <c r="G37" s="24" t="inlineStr">
+        <is>
+          <t>入库</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A38" s="29"/>
+      <c r="B38" s="21" t="n">
+        <v>2</v>
+      </c>
+      <c r="C38" s="21" t="inlineStr">
+        <is>
+          <t>out</t>
+        </is>
+      </c>
+      <c r="D38" s="24" t="inlineStr">
+        <is>
+          <t>出库</t>
+        </is>
+      </c>
+      <c r="E38" s="24" t="inlineStr">
+        <is>
+          <t>OUT</t>
+        </is>
+      </c>
+      <c r="F38" s="24"/>
+      <c r="G38" s="24" t="inlineStr">
+        <is>
+          <t>出库</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A39" s="29"/>
+      <c r="B39" s="21"/>
+      <c r="C39" s="21"/>
+      <c r="D39" s="24"/>
+      <c r="E39" s="24"/>
+      <c r="F39" s="24"/>
+      <c r="G39" s="24"/>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A40" s="29"/>
+      <c r="B40" s="21"/>
+      <c r="C40" s="21"/>
+      <c r="D40" s="24"/>
+      <c r="E40" s="24"/>
+      <c r="F40" s="24"/>
+      <c r="G40" s="24"/>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A41" s="29"/>
+      <c r="B41" s="21"/>
+      <c r="C41" s="21"/>
+      <c r="D41" s="24"/>
+      <c r="E41" s="24"/>
+      <c r="F41" s="24"/>
+      <c r="G41" s="24"/>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A42" s="29"/>
+      <c r="B42" s="21"/>
+      <c r="C42" s="21"/>
+      <c r="D42" s="24"/>
+      <c r="E42" s="24"/>
+      <c r="F42" s="24"/>
+      <c r="G42" s="24"/>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A43" s="29"/>
+      <c r="B43" s="21"/>
+      <c r="C43" s="21"/>
+      <c r="D43" s="24"/>
+      <c r="E43" s="24"/>
+      <c r="F43" s="24"/>
+      <c r="G43" s="24"/>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A44" s="29"/>
+      <c r="B44" s="21"/>
+      <c r="C44" s="25"/>
+      <c r="D44" s="24"/>
+      <c r="E44" s="24"/>
+      <c r="F44" s="24"/>
+      <c r="G44" s="24"/>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A45" s="29"/>
+      <c r="B45" s="26"/>
+      <c r="C45" s="26"/>
+      <c r="D45" s="26"/>
+      <c r="E45" s="26"/>
+      <c r="F45" s="26"/>
+      <c r="G45" s="26"/>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A46" s="29" t="n">
+        <v>4</v>
+      </c>
+      <c r="B46" s="32" t="inlineStr">
+        <is>
+          <t>名称</t>
+        </is>
+      </c>
+      <c r="C46" s="32"/>
+      <c r="D46" s="34" t="inlineStr">
+        <is>
+          <t>checkType</t>
+        </is>
+      </c>
+      <c r="E46" s="34"/>
+      <c r="F46" s="20" t="inlineStr">
+        <is>
+          <t>值类型</t>
+        </is>
+      </c>
+      <c r="G46" s="17"/>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A47" s="29"/>
+      <c r="B47" s="32" t="inlineStr">
+        <is>
+          <t>中文名</t>
+        </is>
+      </c>
+      <c r="C47" s="32"/>
+      <c r="D47" s="34" t="inlineStr">
+        <is>
+          <t>盘库类型</t>
+        </is>
+      </c>
+      <c r="E47" s="34"/>
+      <c r="F47" s="20" t="inlineStr">
+        <is>
+          <t>英文名</t>
+        </is>
+      </c>
+      <c r="G47" s="21"/>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A48" s="29"/>
+      <c r="B48" s="32" t="inlineStr">
+        <is>
+          <t>描述</t>
+        </is>
+      </c>
+      <c r="C48" s="32"/>
+      <c r="D48" s="34" t="inlineStr">
+        <is>
+          <t>盘库类型</t>
+        </is>
+      </c>
+      <c r="E48" s="34"/>
+      <c r="F48" s="34"/>
+      <c r="G48" s="34"/>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A49" s="29"/>
+      <c r="B49" s="37" t="inlineStr">
+        <is>
+          <t>字典项</t>
+        </is>
+      </c>
+      <c r="C49" s="37"/>
+      <c r="D49" s="37"/>
+      <c r="E49" s="37"/>
+      <c r="F49" s="37"/>
+      <c r="G49" s="37"/>
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A50" s="29"/>
+      <c r="B50" s="22" t="inlineStr">
+        <is>
+          <t>序号</t>
+        </is>
+      </c>
+      <c r="C50" s="23" t="inlineStr">
+        <is>
+          <t>值</t>
+        </is>
+      </c>
+      <c r="D50" s="23" t="inlineStr">
+        <is>
+          <t>名称</t>
+        </is>
+      </c>
+      <c r="E50" s="23" t="inlineStr">
+        <is>
+          <t>代码</t>
+        </is>
+      </c>
+      <c r="F50" s="23" t="inlineStr">
+        <is>
+          <t>英文名</t>
+        </is>
+      </c>
+      <c r="G50" s="23" t="inlineStr">
+        <is>
+          <t>描述</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A51" s="29"/>
+      <c r="B51" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="C51" s="21" t="inlineStr">
+        <is>
+          <t>initial</t>
+        </is>
+      </c>
+      <c r="D51" s="24" t="inlineStr">
+        <is>
+          <t>初始盘库</t>
+        </is>
+      </c>
+      <c r="E51" s="24" t="inlineStr">
+        <is>
+          <t>INITIAL</t>
+        </is>
+      </c>
+      <c r="F51" s="24"/>
+      <c r="G51" s="24" t="inlineStr">
+        <is>
+          <t>初始盘库</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A52" s="29"/>
+      <c r="B52" s="21" t="n">
+        <v>2</v>
+      </c>
+      <c r="C52" s="21" t="inlineStr">
+        <is>
+          <t>periodic</t>
+        </is>
+      </c>
+      <c r="D52" s="24" t="inlineStr">
+        <is>
+          <t>定期盘库</t>
+        </is>
+      </c>
+      <c r="E52" s="24" t="inlineStr">
+        <is>
+          <t>PERIODIC</t>
+        </is>
+      </c>
+      <c r="F52" s="24"/>
+      <c r="G52" s="24" t="inlineStr">
+        <is>
+          <t>定期盘库</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A53" s="29"/>
+      <c r="B53" s="21" t="n">
+        <v>3</v>
+      </c>
+      <c r="C53" s="21" t="inlineStr">
+        <is>
+          <t>final</t>
+        </is>
+      </c>
+      <c r="D53" s="24" t="inlineStr">
+        <is>
+          <t>最终盘库</t>
+        </is>
+      </c>
+      <c r="E53" s="24" t="inlineStr">
+        <is>
+          <t>FINAL</t>
+        </is>
+      </c>
+      <c r="F53" s="24"/>
+      <c r="G53" s="24" t="inlineStr">
+        <is>
+          <t>最终盘库</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A54" s="29"/>
+      <c r="B54" s="21"/>
+      <c r="C54" s="21"/>
+      <c r="D54" s="24"/>
+      <c r="E54" s="24"/>
+      <c r="F54" s="24"/>
+      <c r="G54" s="24"/>
+    </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A55" s="29"/>
+      <c r="B55" s="21"/>
+      <c r="C55" s="21"/>
+      <c r="D55" s="24"/>
+      <c r="E55" s="24"/>
+      <c r="F55" s="24"/>
+      <c r="G55" s="24"/>
+    </row>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A56" s="29"/>
+      <c r="B56" s="21"/>
+      <c r="C56" s="21"/>
+      <c r="D56" s="24"/>
+      <c r="E56" s="24"/>
+      <c r="F56" s="24"/>
+      <c r="G56" s="24"/>
+    </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A57" s="29"/>
+      <c r="B57" s="21"/>
+      <c r="C57" s="21"/>
+      <c r="D57" s="24"/>
+      <c r="E57" s="24"/>
+      <c r="F57" s="24"/>
+      <c r="G57" s="24"/>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A58" s="29"/>
+      <c r="B58" s="21"/>
+      <c r="C58" s="21"/>
+      <c r="D58" s="24"/>
+      <c r="E58" s="24"/>
+      <c r="F58" s="24"/>
+      <c r="G58" s="24"/>
+    </row>
+    <row r="59" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A59" s="29"/>
+      <c r="B59" s="21"/>
+      <c r="C59" s="25"/>
+      <c r="D59" s="24"/>
+      <c r="E59" s="24"/>
+      <c r="F59" s="24"/>
+      <c r="G59" s="24"/>
+    </row>
+    <row r="60" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A60" s="29"/>
+      <c r="B60" s="26"/>
+      <c r="C60" s="26"/>
+      <c r="D60" s="26"/>
+      <c r="E60" s="26"/>
+      <c r="F60" s="26"/>
+      <c r="G60" s="26"/>
+    </row>
+    <row r="61" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A61" s="29" t="n">
+        <v>5</v>
+      </c>
+      <c r="B61" s="32" t="inlineStr">
+        <is>
+          <t>名称</t>
+        </is>
+      </c>
+      <c r="C61" s="32"/>
+      <c r="D61" s="34" t="inlineStr">
+        <is>
+          <t>supplierStatus</t>
+        </is>
+      </c>
+      <c r="E61" s="34"/>
+      <c r="F61" s="20" t="inlineStr">
+        <is>
+          <t>值类型</t>
+        </is>
+      </c>
+      <c r="G61" s="17"/>
+    </row>
+    <row r="62" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A62" s="29"/>
+      <c r="B62" s="32" t="inlineStr">
+        <is>
+          <t>中文名</t>
+        </is>
+      </c>
+      <c r="C62" s="32"/>
+      <c r="D62" s="34" t="inlineStr">
+        <is>
+          <t>供应商状态</t>
+        </is>
+      </c>
+      <c r="E62" s="34"/>
+      <c r="F62" s="20" t="inlineStr">
+        <is>
+          <t>英文名</t>
+        </is>
+      </c>
+      <c r="G62" s="21"/>
+    </row>
+    <row r="63" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A63" s="29"/>
+      <c r="B63" s="32" t="inlineStr">
+        <is>
+          <t>描述</t>
+        </is>
+      </c>
+      <c r="C63" s="32"/>
+      <c r="D63" s="34" t="inlineStr">
+        <is>
+          <t>供应商状态</t>
+        </is>
+      </c>
+      <c r="E63" s="34"/>
+      <c r="F63" s="34"/>
+      <c r="G63" s="34"/>
+    </row>
+    <row r="64" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A64" s="29"/>
+      <c r="B64" s="37" t="inlineStr">
+        <is>
+          <t>字典项</t>
+        </is>
+      </c>
+      <c r="C64" s="37"/>
+      <c r="D64" s="37"/>
+      <c r="E64" s="37"/>
+      <c r="F64" s="37"/>
+      <c r="G64" s="37"/>
+    </row>
+    <row r="65" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A65" s="29"/>
+      <c r="B65" s="22" t="inlineStr">
+        <is>
+          <t>序号</t>
+        </is>
+      </c>
+      <c r="C65" s="23" t="inlineStr">
+        <is>
+          <t>值</t>
+        </is>
+      </c>
+      <c r="D65" s="23" t="inlineStr">
+        <is>
+          <t>名称</t>
+        </is>
+      </c>
+      <c r="E65" s="23" t="inlineStr">
+        <is>
+          <t>代码</t>
+        </is>
+      </c>
+      <c r="F65" s="23" t="inlineStr">
+        <is>
+          <t>英文名</t>
+        </is>
+      </c>
+      <c r="G65" s="23" t="inlineStr">
+        <is>
+          <t>描述</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A66" s="29"/>
+      <c r="B66" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="C66" s="21" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="D66" s="24" t="inlineStr">
+        <is>
+          <t>启用</t>
+        </is>
+      </c>
+      <c r="E66" s="24" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="F66" s="24"/>
+      <c r="G66" s="24" t="inlineStr">
+        <is>
+          <t>启用</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A67" s="29"/>
+      <c r="B67" s="21" t="n">
+        <v>2</v>
+      </c>
+      <c r="C67" s="21" t="inlineStr">
+        <is>
+          <t>disabled</t>
+        </is>
+      </c>
+      <c r="D67" s="24" t="inlineStr">
+        <is>
+          <t>禁用</t>
+        </is>
+      </c>
+      <c r="E67" s="24" t="inlineStr">
+        <is>
+          <t>DISABLED</t>
+        </is>
+      </c>
+      <c r="F67" s="24"/>
+      <c r="G67" s="24" t="inlineStr">
+        <is>
+          <t>禁用</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A68" s="29"/>
+      <c r="B68" s="21"/>
+      <c r="C68" s="21"/>
+      <c r="D68" s="24"/>
+      <c r="E68" s="24"/>
+      <c r="F68" s="24"/>
+      <c r="G68" s="24"/>
+    </row>
+    <row r="69" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A69" s="29"/>
+      <c r="B69" s="21"/>
+      <c r="C69" s="21"/>
+      <c r="D69" s="24"/>
+      <c r="E69" s="24"/>
+      <c r="F69" s="24"/>
+      <c r="G69" s="24"/>
+    </row>
+    <row r="70" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A70" s="29"/>
+      <c r="B70" s="21"/>
+      <c r="C70" s="21"/>
+      <c r="D70" s="24"/>
+      <c r="E70" s="24"/>
+      <c r="F70" s="24"/>
+      <c r="G70" s="24"/>
+    </row>
+    <row r="71" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A71" s="29"/>
+      <c r="B71" s="21"/>
+      <c r="C71" s="21"/>
+      <c r="D71" s="24"/>
+      <c r="E71" s="24"/>
+      <c r="F71" s="24"/>
+      <c r="G71" s="24"/>
+    </row>
+    <row r="72" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A72" s="29"/>
+      <c r="B72" s="21"/>
+      <c r="C72" s="21"/>
+      <c r="D72" s="24"/>
+      <c r="E72" s="24"/>
+      <c r="F72" s="24"/>
+      <c r="G72" s="24"/>
+    </row>
+    <row r="73" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A73" s="29"/>
+      <c r="B73" s="21"/>
+      <c r="C73" s="25"/>
+      <c r="D73" s="24"/>
+      <c r="E73" s="24"/>
+      <c r="F73" s="24"/>
+      <c r="G73" s="24"/>
+    </row>
+    <row r="74" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A74" s="29"/>
+      <c r="B74" s="26"/>
+      <c r="C74" s="26"/>
+      <c r="D74" s="26"/>
+      <c r="E74" s="26"/>
+      <c r="F74" s="26"/>
+      <c r="G74" s="26"/>
+    </row>
+    <row r="75" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A75" s="29" t="n">
+        <v>6</v>
+      </c>
+      <c r="B75" s="32" t="inlineStr">
+        <is>
+          <t>名称</t>
+        </is>
+      </c>
+      <c r="C75" s="32"/>
+      <c r="D75" s="34" t="inlineStr">
+        <is>
+          <t>serviceCompanyStatus</t>
+        </is>
+      </c>
+      <c r="E75" s="34"/>
+      <c r="F75" s="20" t="inlineStr">
+        <is>
+          <t>值类型</t>
+        </is>
+      </c>
+      <c r="G75" s="17"/>
+    </row>
+    <row r="76" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A76" s="29"/>
+      <c r="B76" s="32" t="inlineStr">
+        <is>
+          <t>中文名</t>
+        </is>
+      </c>
+      <c r="C76" s="32"/>
+      <c r="D76" s="34" t="inlineStr">
+        <is>
+          <t>服务公司状态</t>
+        </is>
+      </c>
+      <c r="E76" s="34"/>
+      <c r="F76" s="20" t="inlineStr">
+        <is>
+          <t>英文名</t>
+        </is>
+      </c>
+      <c r="G76" s="21"/>
+    </row>
+    <row r="77" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A77" s="29"/>
+      <c r="B77" s="32" t="inlineStr">
+        <is>
+          <t>描述</t>
+        </is>
+      </c>
+      <c r="C77" s="32"/>
+      <c r="D77" s="34" t="inlineStr">
+        <is>
+          <t>服务公司状态</t>
+        </is>
+      </c>
+      <c r="E77" s="34"/>
+      <c r="F77" s="34"/>
+      <c r="G77" s="34"/>
+    </row>
+    <row r="78" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A78" s="29"/>
+      <c r="B78" s="37" t="inlineStr">
+        <is>
+          <t>字典项</t>
+        </is>
+      </c>
+      <c r="C78" s="37"/>
+      <c r="D78" s="37"/>
+      <c r="E78" s="37"/>
+      <c r="F78" s="37"/>
+      <c r="G78" s="37"/>
+    </row>
+    <row r="79" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A79" s="29"/>
+      <c r="B79" s="22" t="inlineStr">
+        <is>
+          <t>序号</t>
+        </is>
+      </c>
+      <c r="C79" s="23" t="inlineStr">
+        <is>
+          <t>值</t>
+        </is>
+      </c>
+      <c r="D79" s="23" t="inlineStr">
+        <is>
+          <t>名称</t>
+        </is>
+      </c>
+      <c r="E79" s="23" t="inlineStr">
+        <is>
+          <t>代码</t>
+        </is>
+      </c>
+      <c r="F79" s="23" t="inlineStr">
+        <is>
+          <t>英文名</t>
+        </is>
+      </c>
+      <c r="G79" s="23" t="inlineStr">
+        <is>
+          <t>描述</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A80" s="29"/>
+      <c r="B80" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="C80" s="21" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="D80" s="24" t="inlineStr">
+        <is>
+          <t>启用</t>
+        </is>
+      </c>
+      <c r="E80" s="24" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="F80" s="24"/>
+      <c r="G80" s="24" t="inlineStr">
+        <is>
+          <t>启用</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A81" s="29"/>
+      <c r="B81" s="21" t="n">
+        <v>2</v>
+      </c>
+      <c r="C81" s="21" t="inlineStr">
+        <is>
+          <t>disabled</t>
+        </is>
+      </c>
+      <c r="D81" s="24" t="inlineStr">
+        <is>
+          <t>禁用</t>
+        </is>
+      </c>
+      <c r="E81" s="24" t="inlineStr">
+        <is>
+          <t>DISABLED</t>
+        </is>
+      </c>
+      <c r="F81" s="24"/>
+      <c r="G81" s="24" t="inlineStr">
+        <is>
+          <t>禁用</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A82" s="29"/>
+      <c r="B82" s="21"/>
+      <c r="C82" s="21"/>
+      <c r="D82" s="24"/>
+      <c r="E82" s="24"/>
+      <c r="F82" s="24"/>
+      <c r="G82" s="24"/>
+    </row>
+    <row r="83" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A83" s="29"/>
+      <c r="B83" s="21"/>
+      <c r="C83" s="21"/>
+      <c r="D83" s="24"/>
+      <c r="E83" s="24"/>
+      <c r="F83" s="24"/>
+      <c r="G83" s="24"/>
+    </row>
+    <row r="84" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A84" s="29"/>
+      <c r="B84" s="21"/>
+      <c r="C84" s="21"/>
+      <c r="D84" s="24"/>
+      <c r="E84" s="24"/>
+      <c r="F84" s="24"/>
+      <c r="G84" s="24"/>
+    </row>
+    <row r="85" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A85" s="29"/>
+      <c r="B85" s="21"/>
+      <c r="C85" s="21"/>
+      <c r="D85" s="24"/>
+      <c r="E85" s="24"/>
+      <c r="F85" s="24"/>
+      <c r="G85" s="24"/>
+    </row>
+    <row r="86" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A86" s="29"/>
+      <c r="B86" s="21"/>
+      <c r="C86" s="21"/>
+      <c r="D86" s="24"/>
+      <c r="E86" s="24"/>
+      <c r="F86" s="24"/>
+      <c r="G86" s="24"/>
+    </row>
+    <row r="87" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A87" s="29"/>
+      <c r="B87" s="21"/>
+      <c r="C87" s="25"/>
+      <c r="D87" s="24"/>
+      <c r="E87" s="24"/>
+      <c r="F87" s="24"/>
+      <c r="G87" s="24"/>
+    </row>
+    <row r="88" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A88" s="29"/>
+      <c r="B88" s="26"/>
+      <c r="C88" s="26"/>
+      <c r="D88" s="26"/>
+      <c r="E88" s="26"/>
+      <c r="F88" s="26"/>
+      <c r="G88" s="26"/>
     </row>
   </sheetData>
-  <mergeCells count="9">
-    <mergeCell ref="A1:A13"/>
+  <mergeCells count="54">
+    <mergeCell ref="A1:A16"/>
     <mergeCell ref="B1:C1"/>
     <mergeCell ref="D1:E1"/>
     <mergeCell ref="B2:C2"/>
@@ -9928,33 +11085,78 @@
     <mergeCell ref="B3:C3"/>
     <mergeCell ref="D3:G3"/>
     <mergeCell ref="B4:G4"/>
-    <mergeCell ref="B13:G13"/>
+    <mergeCell ref="B16:G16"/>
+    <mergeCell ref="A17:A31"/>
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="D17:E17"/>
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="D18:E18"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="D19:G19"/>
+    <mergeCell ref="B20:G20"/>
+    <mergeCell ref="B31:G31"/>
+    <mergeCell ref="A32:A45"/>
+    <mergeCell ref="B32:C32"/>
+    <mergeCell ref="D32:E32"/>
+    <mergeCell ref="B33:C33"/>
+    <mergeCell ref="D33:E33"/>
+    <mergeCell ref="B34:C34"/>
+    <mergeCell ref="D34:G34"/>
+    <mergeCell ref="B35:G35"/>
+    <mergeCell ref="B45:G45"/>
+    <mergeCell ref="A46:A60"/>
+    <mergeCell ref="B46:C46"/>
+    <mergeCell ref="D46:E46"/>
+    <mergeCell ref="B47:C47"/>
+    <mergeCell ref="D47:E47"/>
+    <mergeCell ref="B48:C48"/>
+    <mergeCell ref="D48:G48"/>
+    <mergeCell ref="B49:G49"/>
+    <mergeCell ref="B60:G60"/>
+    <mergeCell ref="A61:A74"/>
+    <mergeCell ref="B61:C61"/>
+    <mergeCell ref="D61:E61"/>
+    <mergeCell ref="B62:C62"/>
+    <mergeCell ref="D62:E62"/>
+    <mergeCell ref="B63:C63"/>
+    <mergeCell ref="D63:G63"/>
+    <mergeCell ref="B64:G64"/>
+    <mergeCell ref="B74:G74"/>
+    <mergeCell ref="A75:A88"/>
+    <mergeCell ref="B75:C75"/>
+    <mergeCell ref="D75:E75"/>
+    <mergeCell ref="B76:C76"/>
+    <mergeCell ref="D76:E76"/>
+    <mergeCell ref="B77:C77"/>
+    <mergeCell ref="D77:G77"/>
+    <mergeCell ref="B78:G78"/>
+    <mergeCell ref="B88:G88"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{eefd2834-e7e3-4c81-acbf-3a2971765552}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:R35"/>
-  <sheetFormatPr defaultRowHeight="14.0" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.33203125" customWidth="1"/>
-    <col min="2" max="2" width="4.4140625" customWidth="1"/>
+    <col min="2" max="2" width="4.44140625" customWidth="1"/>
     <col min="3" max="3" width="5.6640625" customWidth="1"/>
-    <col min="4" max="4" width="12.9140625" customWidth="1"/>
+    <col min="4" max="4" width="12.88671875" customWidth="1"/>
     <col min="5" max="5" width="4.6640625" customWidth="1"/>
-    <col min="6" max="6" width="4.75" customWidth="1"/>
-    <col min="7" max="7" width="15.08203125" customWidth="1"/>
+    <col min="6" max="6" width="4.77734375" customWidth="1"/>
+    <col min="7" max="7" width="15.109375" customWidth="1"/>
     <col min="8" max="8" width="13.0" customWidth="1"/>
     <col min="9" max="9" width="8.5" customWidth="1"/>
-    <col min="10" max="10" width="6.25" customWidth="1"/>
-    <col min="11" max="11" width="4.75" customWidth="1"/>
+    <col min="10" max="10" width="6.21875" customWidth="1"/>
+    <col min="11" max="11" width="4.77734375" customWidth="1"/>
     <col min="12" max="12" width="11.0" customWidth="1"/>
-    <col min="13" max="13" width="6.08203125" customWidth="1"/>
-    <col min="14" max="14" width="8.25" customWidth="1"/>
+    <col min="13" max="13" width="6.109375" customWidth="1"/>
+    <col min="14" max="14" width="8.21875" customWidth="1"/>
     <col min="15" max="15" width="12.6640625" customWidth="1"/>
-    <col min="16" max="16" width="11.08203125" customWidth="1"/>
+    <col min="16" max="16" width="11.109375" customWidth="1"/>
     <col min="17" max="17" width="8.5" customWidth="1"/>
     <col min="18" max="18" width="8.5" customWidth="1"/>
   </cols>
@@ -10040,7 +11242,11 @@
       <c r="F3" s="67"/>
       <c r="G3" s="67"/>
       <c r="H3" s="67"/>
-      <c r="I3" s="5"/>
+      <c r="I3" s="5" t="inlineStr">
+        <is>
+          <t>所属模块</t>
+        </is>
+      </c>
       <c r="J3" s="34"/>
       <c r="K3" s="34"/>
       <c r="L3" s="34"/>
@@ -10146,7 +11352,7 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>属性名</t>
+          <t>控件</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -10230,11 +11436,7 @@
           <t>id</t>
         </is>
       </c>
-      <c r="E8" s="9" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
+      <c r="E8" s="9"/>
       <c r="F8" s="7"/>
       <c r="G8" s="9"/>
       <c r="H8" s="9" t="inlineStr">
@@ -10276,11 +11478,7 @@
           <t>material_name</t>
         </is>
       </c>
-      <c r="E9" s="9" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="E9" s="9"/>
       <c r="F9" s="7"/>
       <c r="G9" s="9"/>
       <c r="H9" s="9" t="inlineStr">
@@ -10322,11 +11520,7 @@
           <t>unit</t>
         </is>
       </c>
-      <c r="E10" s="9" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="E10" s="9"/>
       <c r="F10" s="7"/>
       <c r="G10" s="9"/>
       <c r="H10" s="9" t="inlineStr">
@@ -10372,11 +11566,7 @@
           <t>specification</t>
         </is>
       </c>
-      <c r="E11" s="9" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="E11" s="9"/>
       <c r="F11" s="7"/>
       <c r="G11" s="9"/>
       <c r="H11" s="9" t="inlineStr">
@@ -10418,11 +11608,7 @@
           <t>material_image</t>
         </is>
       </c>
-      <c r="E12" s="9" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="E12" s="9"/>
       <c r="F12" s="7"/>
       <c r="G12" s="9"/>
       <c r="H12" s="9" t="inlineStr">
@@ -10464,11 +11650,7 @@
           <t>brand</t>
         </is>
       </c>
-      <c r="E13" s="9" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="E13" s="9"/>
       <c r="F13" s="7"/>
       <c r="G13" s="9"/>
       <c r="H13" s="9" t="inlineStr">
@@ -10510,11 +11692,7 @@
           <t>remark</t>
         </is>
       </c>
-      <c r="E14" s="9" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="E14" s="9"/>
       <c r="F14" s="7"/>
       <c r="G14" s="9"/>
       <c r="H14" s="9" t="inlineStr">
@@ -10738,9 +11916,7 @@
         </is>
       </c>
       <c r="N21" s="60"/>
-      <c r="O21" s="41" t="b">
-        <v>0</v>
-      </c>
+      <c r="O21" s="41"/>
       <c r="P21" s="41"/>
       <c r="Q21" s="41"/>
       <c r="R21" s="41"/>
@@ -11215,26 +12391,26 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{dcf824d0-f9f2-466b-b09e-bda6b592498c}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:R36"/>
-  <sheetFormatPr defaultRowHeight="14.0" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.33203125" customWidth="1"/>
-    <col min="2" max="2" width="4.4140625" customWidth="1"/>
+    <col min="2" max="2" width="4.44140625" customWidth="1"/>
     <col min="3" max="3" width="5.6640625" customWidth="1"/>
-    <col min="4" max="4" width="12.9140625" customWidth="1"/>
+    <col min="4" max="4" width="12.88671875" customWidth="1"/>
     <col min="5" max="5" width="4.6640625" customWidth="1"/>
-    <col min="6" max="6" width="4.75" customWidth="1"/>
-    <col min="7" max="7" width="15.08203125" customWidth="1"/>
+    <col min="6" max="6" width="4.77734375" customWidth="1"/>
+    <col min="7" max="7" width="15.109375" customWidth="1"/>
     <col min="8" max="8" width="13.0" customWidth="1"/>
     <col min="9" max="9" width="8.5" customWidth="1"/>
-    <col min="10" max="10" width="6.25" customWidth="1"/>
-    <col min="11" max="11" width="4.75" customWidth="1"/>
+    <col min="10" max="10" width="6.21875" customWidth="1"/>
+    <col min="11" max="11" width="4.77734375" customWidth="1"/>
     <col min="12" max="12" width="11.0" customWidth="1"/>
-    <col min="13" max="13" width="6.08203125" customWidth="1"/>
-    <col min="14" max="14" width="8.25" customWidth="1"/>
+    <col min="13" max="13" width="6.109375" customWidth="1"/>
+    <col min="14" max="14" width="8.21875" customWidth="1"/>
     <col min="15" max="15" width="12.6640625" customWidth="1"/>
-    <col min="16" max="16" width="11.08203125" customWidth="1"/>
+    <col min="16" max="16" width="11.109375" customWidth="1"/>
     <col min="17" max="17" width="8.5" customWidth="1"/>
     <col min="18" max="18" width="8.5" customWidth="1"/>
   </cols>
@@ -11320,7 +12496,11 @@
       <c r="F3" s="67"/>
       <c r="G3" s="67"/>
       <c r="H3" s="67"/>
-      <c r="I3" s="5"/>
+      <c r="I3" s="5" t="inlineStr">
+        <is>
+          <t>所属模块</t>
+        </is>
+      </c>
       <c r="J3" s="34"/>
       <c r="K3" s="34"/>
       <c r="L3" s="34"/>
@@ -11426,7 +12606,7 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>属性名</t>
+          <t>控件</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -11510,11 +12690,7 @@
           <t>id</t>
         </is>
       </c>
-      <c r="E8" s="9" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
+      <c r="E8" s="9"/>
       <c r="F8" s="7"/>
       <c r="G8" s="9"/>
       <c r="H8" s="9" t="inlineStr">
@@ -11556,11 +12732,7 @@
           <t>supplier_name</t>
         </is>
       </c>
-      <c r="E9" s="9" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="E9" s="9"/>
       <c r="F9" s="7"/>
       <c r="G9" s="9"/>
       <c r="H9" s="9" t="inlineStr">
@@ -11602,11 +12774,7 @@
           <t>social_credit_code</t>
         </is>
       </c>
-      <c r="E10" s="9" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="E10" s="9"/>
       <c r="F10" s="7"/>
       <c r="G10" s="9"/>
       <c r="H10" s="9" t="inlineStr">
@@ -11648,11 +12816,7 @@
           <t>food_safety_cert</t>
         </is>
       </c>
-      <c r="E11" s="9" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="E11" s="9"/>
       <c r="F11" s="7"/>
       <c r="G11" s="9"/>
       <c r="H11" s="9" t="inlineStr">
@@ -11694,11 +12858,7 @@
           <t>contact_info</t>
         </is>
       </c>
-      <c r="E12" s="9" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="E12" s="9"/>
       <c r="F12" s="7"/>
       <c r="G12" s="9"/>
       <c r="H12" s="9" t="inlineStr">
@@ -11740,11 +12900,7 @@
           <t>company_profile</t>
         </is>
       </c>
-      <c r="E13" s="9" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="E13" s="9"/>
       <c r="F13" s="7"/>
       <c r="G13" s="9"/>
       <c r="H13" s="9" t="inlineStr">
@@ -11786,11 +12942,7 @@
           <t>remark</t>
         </is>
       </c>
-      <c r="E14" s="9" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="E14" s="9"/>
       <c r="F14" s="7"/>
       <c r="G14" s="9"/>
       <c r="H14" s="9" t="inlineStr">
@@ -11832,11 +12984,7 @@
           <t>status</t>
         </is>
       </c>
-      <c r="E15" s="9" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="E15" s="9"/>
       <c r="F15" s="7"/>
       <c r="G15" s="9"/>
       <c r="H15" s="9" t="inlineStr">
@@ -12064,9 +13212,7 @@
         </is>
       </c>
       <c r="N22" s="60"/>
-      <c r="O22" s="41" t="b">
-        <v>0</v>
-      </c>
+      <c r="O22" s="41"/>
       <c r="P22" s="41"/>
       <c r="Q22" s="41"/>
       <c r="R22" s="41"/>
@@ -12541,26 +13687,26 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{77617f76-e093-43d3-9ec0-10fe65e9dbff}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:R44"/>
-  <sheetFormatPr defaultRowHeight="14.0" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.33203125" customWidth="1"/>
-    <col min="2" max="2" width="4.4140625" customWidth="1"/>
+    <col min="2" max="2" width="4.44140625" customWidth="1"/>
     <col min="3" max="3" width="5.6640625" customWidth="1"/>
-    <col min="4" max="4" width="12.9140625" customWidth="1"/>
+    <col min="4" max="4" width="12.88671875" customWidth="1"/>
     <col min="5" max="5" width="4.6640625" customWidth="1"/>
-    <col min="6" max="6" width="4.75" customWidth="1"/>
-    <col min="7" max="7" width="15.08203125" customWidth="1"/>
+    <col min="6" max="6" width="4.77734375" customWidth="1"/>
+    <col min="7" max="7" width="15.109375" customWidth="1"/>
     <col min="8" max="8" width="13.0" customWidth="1"/>
     <col min="9" max="9" width="8.5" customWidth="1"/>
-    <col min="10" max="10" width="6.25" customWidth="1"/>
-    <col min="11" max="11" width="4.75" customWidth="1"/>
+    <col min="10" max="10" width="6.21875" customWidth="1"/>
+    <col min="11" max="11" width="4.77734375" customWidth="1"/>
     <col min="12" max="12" width="11.0" customWidth="1"/>
-    <col min="13" max="13" width="6.08203125" customWidth="1"/>
-    <col min="14" max="14" width="8.25" customWidth="1"/>
+    <col min="13" max="13" width="6.109375" customWidth="1"/>
+    <col min="14" max="14" width="8.21875" customWidth="1"/>
     <col min="15" max="15" width="12.6640625" customWidth="1"/>
-    <col min="16" max="16" width="11.08203125" customWidth="1"/>
+    <col min="16" max="16" width="11.109375" customWidth="1"/>
     <col min="17" max="17" width="8.5" customWidth="1"/>
     <col min="18" max="18" width="8.5" customWidth="1"/>
   </cols>
@@ -12646,7 +13792,11 @@
       <c r="F3" s="67"/>
       <c r="G3" s="67"/>
       <c r="H3" s="67"/>
-      <c r="I3" s="5"/>
+      <c r="I3" s="5" t="inlineStr">
+        <is>
+          <t>所属模块</t>
+        </is>
+      </c>
       <c r="J3" s="34"/>
       <c r="K3" s="34"/>
       <c r="L3" s="34"/>
@@ -12752,7 +13902,7 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>属性名</t>
+          <t>控件</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -12836,11 +13986,7 @@
           <t>id</t>
         </is>
       </c>
-      <c r="E8" s="9" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
+      <c r="E8" s="9"/>
       <c r="F8" s="7"/>
       <c r="G8" s="9"/>
       <c r="H8" s="9" t="inlineStr">
@@ -12882,11 +14028,7 @@
           <t>company_name</t>
         </is>
       </c>
-      <c r="E9" s="9" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="E9" s="9"/>
       <c r="F9" s="7"/>
       <c r="G9" s="9"/>
       <c r="H9" s="9" t="inlineStr">
@@ -12928,11 +14070,7 @@
           <t>social_credit_code</t>
         </is>
       </c>
-      <c r="E10" s="9" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="E10" s="9"/>
       <c r="F10" s="7"/>
       <c r="G10" s="9"/>
       <c r="H10" s="9" t="inlineStr">
@@ -12974,11 +14112,7 @@
           <t>food_safety_cert</t>
         </is>
       </c>
-      <c r="E11" s="9" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="E11" s="9"/>
       <c r="F11" s="7"/>
       <c r="G11" s="9"/>
       <c r="H11" s="9" t="inlineStr">
@@ -13020,11 +14154,7 @@
           <t>contact_info</t>
         </is>
       </c>
-      <c r="E12" s="9" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="E12" s="9"/>
       <c r="F12" s="7"/>
       <c r="G12" s="9"/>
       <c r="H12" s="9" t="inlineStr">
@@ -13066,11 +14196,7 @@
           <t>company_profile</t>
         </is>
       </c>
-      <c r="E13" s="9" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="E13" s="9"/>
       <c r="F13" s="7"/>
       <c r="G13" s="9"/>
       <c r="H13" s="9" t="inlineStr">
@@ -13112,11 +14238,7 @@
           <t>remark</t>
         </is>
       </c>
-      <c r="E14" s="9" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="E14" s="9"/>
       <c r="F14" s="7"/>
       <c r="G14" s="9"/>
       <c r="H14" s="9" t="inlineStr">
@@ -13158,11 +14280,7 @@
           <t>status</t>
         </is>
       </c>
-      <c r="E15" s="9" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="E15" s="9"/>
       <c r="F15" s="7"/>
       <c r="G15" s="9"/>
       <c r="H15" s="9" t="inlineStr">
@@ -13390,9 +14508,7 @@
         </is>
       </c>
       <c r="N22" s="60"/>
-      <c r="O22" s="41" t="b">
-        <v>0</v>
-      </c>
+      <c r="O22" s="41"/>
       <c r="P22" s="41"/>
       <c r="Q22" s="41"/>
       <c r="R22" s="41"/>
@@ -13656,9 +14772,7 @@
         </is>
       </c>
       <c r="N30" s="60"/>
-      <c r="O30" s="41" t="b">
-        <v>0</v>
-      </c>
+      <c r="O30" s="41"/>
       <c r="P30" s="41"/>
       <c r="Q30" s="41"/>
       <c r="R30" s="41"/>
@@ -14170,26 +15284,26 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{147ece0c-727c-4144-bd79-23f8598b5f73}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:R34"/>
-  <sheetFormatPr defaultRowHeight="14.0" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.33203125" customWidth="1"/>
-    <col min="2" max="2" width="4.4140625" customWidth="1"/>
+    <col min="2" max="2" width="4.44140625" customWidth="1"/>
     <col min="3" max="3" width="5.6640625" customWidth="1"/>
-    <col min="4" max="4" width="12.9140625" customWidth="1"/>
+    <col min="4" max="4" width="12.88671875" customWidth="1"/>
     <col min="5" max="5" width="4.6640625" customWidth="1"/>
-    <col min="6" max="6" width="4.75" customWidth="1"/>
-    <col min="7" max="7" width="15.08203125" customWidth="1"/>
+    <col min="6" max="6" width="4.77734375" customWidth="1"/>
+    <col min="7" max="7" width="15.109375" customWidth="1"/>
     <col min="8" max="8" width="13.0" customWidth="1"/>
     <col min="9" max="9" width="8.5" customWidth="1"/>
-    <col min="10" max="10" width="6.25" customWidth="1"/>
-    <col min="11" max="11" width="4.75" customWidth="1"/>
+    <col min="10" max="10" width="6.21875" customWidth="1"/>
+    <col min="11" max="11" width="4.77734375" customWidth="1"/>
     <col min="12" max="12" width="11.0" customWidth="1"/>
-    <col min="13" max="13" width="6.08203125" customWidth="1"/>
-    <col min="14" max="14" width="8.25" customWidth="1"/>
+    <col min="13" max="13" width="6.109375" customWidth="1"/>
+    <col min="14" max="14" width="8.21875" customWidth="1"/>
     <col min="15" max="15" width="12.6640625" customWidth="1"/>
-    <col min="16" max="16" width="11.08203125" customWidth="1"/>
+    <col min="16" max="16" width="11.109375" customWidth="1"/>
     <col min="17" max="17" width="8.5" customWidth="1"/>
     <col min="18" max="18" width="8.5" customWidth="1"/>
   </cols>
@@ -14275,7 +15389,11 @@
       <c r="F3" s="67"/>
       <c r="G3" s="67"/>
       <c r="H3" s="67"/>
-      <c r="I3" s="5"/>
+      <c r="I3" s="5" t="inlineStr">
+        <is>
+          <t>所属模块</t>
+        </is>
+      </c>
       <c r="J3" s="34"/>
       <c r="K3" s="34"/>
       <c r="L3" s="34"/>
@@ -14381,7 +15499,7 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>属性名</t>
+          <t>控件</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -14465,11 +15583,7 @@
           <t>id</t>
         </is>
       </c>
-      <c r="E8" s="9" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
+      <c r="E8" s="9"/>
       <c r="F8" s="7"/>
       <c r="G8" s="9"/>
       <c r="H8" s="9" t="inlineStr">
@@ -14511,11 +15625,7 @@
           <t>menu_name</t>
         </is>
       </c>
-      <c r="E9" s="9" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="E9" s="9"/>
       <c r="F9" s="7"/>
       <c r="G9" s="9"/>
       <c r="H9" s="9" t="inlineStr">
@@ -14557,11 +15667,7 @@
           <t>menu_type</t>
         </is>
       </c>
-      <c r="E10" s="9" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="E10" s="9"/>
       <c r="F10" s="7"/>
       <c r="G10" s="9"/>
       <c r="H10" s="9" t="inlineStr">
@@ -14607,11 +15713,7 @@
           <t>menu_image</t>
         </is>
       </c>
-      <c r="E11" s="9" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="E11" s="9"/>
       <c r="F11" s="7"/>
       <c r="G11" s="9"/>
       <c r="H11" s="9" t="inlineStr">
@@ -14653,11 +15755,7 @@
           <t>ingredients</t>
         </is>
       </c>
-      <c r="E12" s="9" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="E12" s="9"/>
       <c r="F12" s="7"/>
       <c r="G12" s="9"/>
       <c r="H12" s="9" t="inlineStr">
@@ -14699,11 +15797,7 @@
           <t>remark</t>
         </is>
       </c>
-      <c r="E13" s="9" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="E13" s="9"/>
       <c r="F13" s="7"/>
       <c r="G13" s="9"/>
       <c r="H13" s="9" t="inlineStr">
@@ -14927,9 +16021,7 @@
         </is>
       </c>
       <c r="N20" s="60"/>
-      <c r="O20" s="41" t="b">
-        <v>0</v>
-      </c>
+      <c r="O20" s="41"/>
       <c r="P20" s="41"/>
       <c r="Q20" s="41"/>
       <c r="R20" s="41"/>
@@ -15404,26 +16496,26 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6be4e80e-f825-4e04-9b19-e2559e506ae5}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:R34"/>
-  <sheetFormatPr defaultRowHeight="14.0" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.33203125" customWidth="1"/>
-    <col min="2" max="2" width="4.4140625" customWidth="1"/>
+    <col min="2" max="2" width="4.44140625" customWidth="1"/>
     <col min="3" max="3" width="5.6640625" customWidth="1"/>
-    <col min="4" max="4" width="12.9140625" customWidth="1"/>
+    <col min="4" max="4" width="12.88671875" customWidth="1"/>
     <col min="5" max="5" width="4.6640625" customWidth="1"/>
-    <col min="6" max="6" width="4.75" customWidth="1"/>
-    <col min="7" max="7" width="15.08203125" customWidth="1"/>
+    <col min="6" max="6" width="4.77734375" customWidth="1"/>
+    <col min="7" max="7" width="15.109375" customWidth="1"/>
     <col min="8" max="8" width="13.0" customWidth="1"/>
     <col min="9" max="9" width="8.5" customWidth="1"/>
-    <col min="10" max="10" width="6.25" customWidth="1"/>
-    <col min="11" max="11" width="4.75" customWidth="1"/>
+    <col min="10" max="10" width="6.21875" customWidth="1"/>
+    <col min="11" max="11" width="4.77734375" customWidth="1"/>
     <col min="12" max="12" width="11.0" customWidth="1"/>
-    <col min="13" max="13" width="6.08203125" customWidth="1"/>
-    <col min="14" max="14" width="8.25" customWidth="1"/>
+    <col min="13" max="13" width="6.109375" customWidth="1"/>
+    <col min="14" max="14" width="8.21875" customWidth="1"/>
     <col min="15" max="15" width="12.6640625" customWidth="1"/>
-    <col min="16" max="16" width="11.08203125" customWidth="1"/>
+    <col min="16" max="16" width="11.109375" customWidth="1"/>
     <col min="17" max="17" width="8.5" customWidth="1"/>
     <col min="18" max="18" width="8.5" customWidth="1"/>
   </cols>
@@ -15509,7 +16601,11 @@
       <c r="F3" s="67"/>
       <c r="G3" s="67"/>
       <c r="H3" s="67"/>
-      <c r="I3" s="5"/>
+      <c r="I3" s="5" t="inlineStr">
+        <is>
+          <t>所属模块</t>
+        </is>
+      </c>
       <c r="J3" s="34"/>
       <c r="K3" s="34"/>
       <c r="L3" s="34"/>
@@ -15615,7 +16711,7 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>属性名</t>
+          <t>控件</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -15699,11 +16795,7 @@
           <t>id</t>
         </is>
       </c>
-      <c r="E8" s="9" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
+      <c r="E8" s="9"/>
       <c r="F8" s="7"/>
       <c r="G8" s="9"/>
       <c r="H8" s="9" t="inlineStr">
@@ -15745,11 +16837,7 @@
           <t>menu_id</t>
         </is>
       </c>
-      <c r="E9" s="9" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="E9" s="9"/>
       <c r="F9" s="7"/>
       <c r="G9" s="9"/>
       <c r="H9" s="9" t="inlineStr">
@@ -15791,11 +16879,7 @@
           <t>menu_name</t>
         </is>
       </c>
-      <c r="E10" s="9" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="E10" s="9"/>
       <c r="F10" s="7"/>
       <c r="G10" s="9"/>
       <c r="H10" s="9" t="inlineStr">
@@ -15837,11 +16921,7 @@
           <t>menu_image</t>
         </is>
       </c>
-      <c r="E11" s="9" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="E11" s="9"/>
       <c r="F11" s="7"/>
       <c r="G11" s="9"/>
       <c r="H11" s="9" t="inlineStr">
@@ -15883,11 +16963,7 @@
           <t>ingredients</t>
         </is>
       </c>
-      <c r="E12" s="9" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="E12" s="9"/>
       <c r="F12" s="7"/>
       <c r="G12" s="9"/>
       <c r="H12" s="9" t="inlineStr">
@@ -15927,11 +17003,7 @@
       </c>
       <c r="C13" s="7"/>
       <c r="D13" s="9"/>
-      <c r="E13" s="9" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="E13" s="9"/>
       <c r="F13" s="7"/>
       <c r="G13" s="9"/>
       <c r="H13" s="9"/>

</xml_diff>